<commit_message>
voucher itinerary adjustents WIP
</commit_message>
<xml_diff>
--- a/Template/Voucher Template - 1.xlsx
+++ b/Template/Voucher Template - 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Smart Travel PC\Desktop\Vouchers Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5AAC36C-D2B1-4945-84ED-CC6434723928}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{947AFE7B-378D-410B-8C71-DED5DD627394}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="555" windowWidth="18150" windowHeight="15645" xr2:uid="{46FCF62E-0F38-40EF-B40B-6239A54C7BFA}"/>
+    <workbookView xWindow="390" yWindow="330" windowWidth="16650" windowHeight="15870" xr2:uid="{46FCF62E-0F38-40EF-B40B-6239A54C7BFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>TO:</t>
   </si>
@@ -109,16 +109,13 @@
   </si>
   <si>
     <t>*** It will be subject to change based on the local situation ***</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -182,6 +179,18 @@
       <name val="Bahnschrift"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Bahnschrift"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Bahnschrift"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -384,7 +393,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -433,13 +442,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -466,13 +475,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -499,31 +508,25 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -544,13 +547,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -621,61 +624,55 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1076,13 +1073,13 @@
       <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="54" t="s">
+      <c r="A2" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="58"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="56"/>
       <c r="F2" s="13"/>
       <c r="G2" s="14"/>
       <c r="H2" s="15" t="s">
@@ -1094,19 +1091,19 @@
       <c r="N2" s="2"/>
     </row>
     <row r="3" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="94" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="46"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
+      <c r="G3" s="95"/>
+      <c r="H3" s="95"/>
+      <c r="I3" s="95"/>
+      <c r="J3" s="95"/>
+      <c r="K3" s="96"/>
       <c r="N3" s="2"/>
     </row>
     <row r="4" spans="1:14" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1127,52 +1124,52 @@
       <c r="A5" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="50"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="52" t="s">
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="53"/>
-      <c r="H5" s="47"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="49"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="46"/>
+      <c r="J5" s="46"/>
+      <c r="K5" s="47"/>
     </row>
     <row r="6" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="50"/>
-      <c r="C6" s="50"/>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="52" t="s">
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="53"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="49"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="45"/>
+      <c r="I6" s="46"/>
+      <c r="J6" s="46"/>
+      <c r="K6" s="47"/>
     </row>
     <row r="7" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="51"/>
-      <c r="C7" s="51"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="52" t="s">
+      <c r="B7" s="49"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="53"/>
-      <c r="H7" s="47"/>
-      <c r="I7" s="48"/>
-      <c r="J7" s="48"/>
-      <c r="K7" s="49"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="45"/>
+      <c r="I7" s="46"/>
+      <c r="J7" s="46"/>
+      <c r="K7" s="47"/>
     </row>
     <row r="8" spans="1:14" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
@@ -1217,104 +1214,102 @@
     </row>
     <row r="11" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="44"/>
-      <c r="B11" s="72"/>
-      <c r="C11" s="69" t="s">
+      <c r="B11" s="70"/>
+      <c r="C11" s="67" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="71"/>
+      <c r="D11" s="69"/>
       <c r="E11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="59" t="s">
+      <c r="F11" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="59"/>
-      <c r="H11" s="69" t="s">
+      <c r="G11" s="57"/>
+      <c r="H11" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="I11" s="70"/>
-      <c r="J11" s="70"/>
-      <c r="K11" s="71"/>
-    </row>
-    <row r="12" spans="1:14" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="73"/>
-      <c r="B12" s="74"/>
-      <c r="C12" s="85"/>
-      <c r="D12" s="86"/>
-      <c r="E12" s="79"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="62"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="61"/>
-      <c r="J12" s="61"/>
-      <c r="K12" s="62"/>
-    </row>
-    <row r="13" spans="1:14" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="75"/>
-      <c r="B13" s="76"/>
-      <c r="C13" s="87"/>
-      <c r="D13" s="88"/>
-      <c r="E13" s="80"/>
-      <c r="F13" s="63"/>
-      <c r="G13" s="65"/>
-      <c r="H13" s="63"/>
-      <c r="I13" s="64"/>
-      <c r="J13" s="64"/>
-      <c r="K13" s="65"/>
-    </row>
-    <row r="14" spans="1:14" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="75"/>
-      <c r="B14" s="76"/>
-      <c r="C14" s="82" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="83"/>
-      <c r="E14" s="80"/>
-      <c r="F14" s="63"/>
-      <c r="G14" s="65"/>
-      <c r="H14" s="66"/>
-      <c r="I14" s="67"/>
-      <c r="J14" s="67"/>
-      <c r="K14" s="68"/>
-    </row>
-    <row r="15" spans="1:14" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="75"/>
-      <c r="B15" s="76"/>
-      <c r="C15" s="84"/>
-      <c r="D15" s="83"/>
-      <c r="E15" s="80"/>
-      <c r="F15" s="63"/>
-      <c r="G15" s="65"/>
-      <c r="H15" s="60"/>
-      <c r="I15" s="61"/>
-      <c r="J15" s="61"/>
-      <c r="K15" s="62"/>
-    </row>
-    <row r="16" spans="1:14" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="75"/>
-      <c r="B16" s="76"/>
-      <c r="C16" s="87"/>
-      <c r="D16" s="88"/>
-      <c r="E16" s="80"/>
-      <c r="F16" s="63"/>
-      <c r="G16" s="65"/>
-      <c r="H16" s="63"/>
-      <c r="I16" s="64"/>
-      <c r="J16" s="64"/>
-      <c r="K16" s="65"/>
-    </row>
-    <row r="17" spans="1:11" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="77"/>
-      <c r="B17" s="78"/>
-      <c r="C17" s="89"/>
-      <c r="D17" s="90"/>
-      <c r="E17" s="81"/>
-      <c r="F17" s="66"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="66"/>
-      <c r="I17" s="67"/>
-      <c r="J17" s="67"/>
-      <c r="K17" s="68"/>
+      <c r="I11" s="68"/>
+      <c r="J11" s="68"/>
+      <c r="K11" s="69"/>
+    </row>
+    <row r="12" spans="1:14" s="4" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="71"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="86"/>
+      <c r="D12" s="87"/>
+      <c r="E12" s="77"/>
+      <c r="F12" s="58"/>
+      <c r="G12" s="60"/>
+      <c r="H12" s="58"/>
+      <c r="I12" s="59"/>
+      <c r="J12" s="59"/>
+      <c r="K12" s="60"/>
+    </row>
+    <row r="13" spans="1:14" s="4" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="73"/>
+      <c r="B13" s="74"/>
+      <c r="C13" s="88"/>
+      <c r="D13" s="89"/>
+      <c r="E13" s="78"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="63"/>
+      <c r="H13" s="61"/>
+      <c r="I13" s="62"/>
+      <c r="J13" s="62"/>
+      <c r="K13" s="63"/>
+    </row>
+    <row r="14" spans="1:14" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="73"/>
+      <c r="B14" s="74"/>
+      <c r="C14" s="88"/>
+      <c r="D14" s="89"/>
+      <c r="E14" s="78"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="63"/>
+      <c r="H14" s="64"/>
+      <c r="I14" s="65"/>
+      <c r="J14" s="65"/>
+      <c r="K14" s="66"/>
+    </row>
+    <row r="15" spans="1:14" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="73"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="90"/>
+      <c r="D15" s="91"/>
+      <c r="E15" s="78"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="58"/>
+      <c r="I15" s="59"/>
+      <c r="J15" s="59"/>
+      <c r="K15" s="60"/>
+    </row>
+    <row r="16" spans="1:14" s="4" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="73"/>
+      <c r="B16" s="74"/>
+      <c r="C16" s="90"/>
+      <c r="D16" s="91"/>
+      <c r="E16" s="78"/>
+      <c r="F16" s="61"/>
+      <c r="G16" s="63"/>
+      <c r="H16" s="61"/>
+      <c r="I16" s="62"/>
+      <c r="J16" s="62"/>
+      <c r="K16" s="63"/>
+    </row>
+    <row r="17" spans="1:11" s="4" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="75"/>
+      <c r="B17" s="76"/>
+      <c r="C17" s="92"/>
+      <c r="D17" s="93"/>
+      <c r="E17" s="79"/>
+      <c r="F17" s="64"/>
+      <c r="G17" s="66"/>
+      <c r="H17" s="64"/>
+      <c r="I17" s="65"/>
+      <c r="J17" s="65"/>
+      <c r="K17" s="66"/>
     </row>
     <row r="18" spans="1:11" customFormat="1" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1359,10 +1354,10 @@
         <v>22</v>
       </c>
       <c r="G21" s="22"/>
-      <c r="H21" s="100" t="s">
+      <c r="H21" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="I21" s="100"/>
+      <c r="I21" s="85"/>
       <c r="J21" s="22" t="s">
         <v>23</v>
       </c>
@@ -1376,12 +1371,12 @@
       </c>
       <c r="D22" s="40"/>
       <c r="E22" s="11"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="47"/>
-      <c r="H22" s="49"/>
-      <c r="I22" s="47"/>
-      <c r="J22" s="49"/>
-      <c r="K22" s="97"/>
+      <c r="F22" s="83"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="83"/>
+      <c r="I22" s="84"/>
+      <c r="J22" s="83"/>
+      <c r="K22" s="80"/>
     </row>
     <row r="23" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="37"/>
@@ -1391,12 +1386,12 @@
       </c>
       <c r="D23" s="40"/>
       <c r="E23" s="11"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="47"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="47"/>
-      <c r="J23" s="49"/>
-      <c r="K23" s="97"/>
+      <c r="F23" s="83"/>
+      <c r="G23" s="84"/>
+      <c r="H23" s="83"/>
+      <c r="I23" s="84"/>
+      <c r="J23" s="83"/>
+      <c r="K23" s="80"/>
     </row>
     <row r="24" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="22" t="s">
@@ -1407,10 +1402,10 @@
         <v>4</v>
       </c>
       <c r="D24" s="22"/>
-      <c r="E24" s="99" t="s">
+      <c r="E24" s="82" t="s">
         <v>24</v>
       </c>
-      <c r="F24" s="99"/>
+      <c r="F24" s="82"/>
       <c r="G24" s="22" t="s">
         <v>17</v>
       </c>
@@ -1422,28 +1417,28 @@
     <row r="25" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="25"/>
       <c r="B25" s="25"/>
-      <c r="C25" s="97"/>
-      <c r="D25" s="97"/>
-      <c r="E25" s="98"/>
-      <c r="F25" s="98"/>
-      <c r="G25" s="97"/>
-      <c r="H25" s="97"/>
-      <c r="I25" s="97"/>
-      <c r="J25" s="97"/>
-      <c r="K25" s="97"/>
+      <c r="C25" s="80"/>
+      <c r="D25" s="80"/>
+      <c r="E25" s="81"/>
+      <c r="F25" s="81"/>
+      <c r="G25" s="80"/>
+      <c r="H25" s="80"/>
+      <c r="I25" s="80"/>
+      <c r="J25" s="80"/>
+      <c r="K25" s="80"/>
     </row>
     <row r="26" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="25"/>
       <c r="B26" s="25"/>
-      <c r="C26" s="97"/>
-      <c r="D26" s="97"/>
-      <c r="E26" s="98"/>
-      <c r="F26" s="98"/>
-      <c r="G26" s="97"/>
-      <c r="H26" s="97"/>
-      <c r="I26" s="97"/>
-      <c r="J26" s="97"/>
-      <c r="K26" s="97"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="81"/>
+      <c r="F26" s="81"/>
+      <c r="G26" s="80"/>
+      <c r="H26" s="80"/>
+      <c r="I26" s="80"/>
+      <c r="J26" s="80"/>
+      <c r="K26" s="80"/>
     </row>
     <row r="27" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="22" t="s">
@@ -1463,41 +1458,41 @@
     <row r="28" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
-      <c r="C28" s="91"/>
-      <c r="D28" s="92"/>
-      <c r="E28" s="92"/>
-      <c r="F28" s="92"/>
-      <c r="G28" s="92"/>
-      <c r="H28" s="92"/>
-      <c r="I28" s="92"/>
-      <c r="J28" s="92"/>
-      <c r="K28" s="93"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="21"/>
     </row>
     <row r="29" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="22"/>
       <c r="B29" s="22"/>
-      <c r="C29" s="91"/>
-      <c r="D29" s="92"/>
-      <c r="E29" s="92"/>
-      <c r="F29" s="92"/>
-      <c r="G29" s="92"/>
-      <c r="H29" s="92"/>
-      <c r="I29" s="92"/>
-      <c r="J29" s="92"/>
-      <c r="K29" s="93"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="20"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="21"/>
     </row>
     <row r="30" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="22"/>
       <c r="B30" s="22"/>
-      <c r="C30" s="94"/>
-      <c r="D30" s="95"/>
-      <c r="E30" s="95"/>
-      <c r="F30" s="95"/>
-      <c r="G30" s="95"/>
-      <c r="H30" s="95"/>
-      <c r="I30" s="95"/>
-      <c r="J30" s="95"/>
-      <c r="K30" s="96"/>
+      <c r="C30" s="30"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="31"/>
+      <c r="J30" s="31"/>
+      <c r="K30" s="32"/>
     </row>
     <row r="31" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="22" t="s">
@@ -1584,7 +1579,7 @@
       <c r="K36" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="61">
+  <mergeCells count="60">
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H22:I22"/>
@@ -1607,9 +1602,8 @@
     <mergeCell ref="A12:B17"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="E12:E17"/>
-    <mergeCell ref="C14:D15"/>
-    <mergeCell ref="C12:D13"/>
-    <mergeCell ref="C16:D17"/>
+    <mergeCell ref="C12:D14"/>
+    <mergeCell ref="C15:D17"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="H12:K14"/>
     <mergeCell ref="H11:K11"/>

</xml_diff>

<commit_message>
ITINERARY AND VOUCHER DB
</commit_message>
<xml_diff>
--- a/Template/Voucher Template - 1.xlsx
+++ b/Template/Voucher Template - 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Smart Travel PC\Desktop\Vouchers Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{947AFE7B-378D-410B-8C71-DED5DD627394}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF7E66CA-C187-4E00-B33E-A5BB49791B84}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="330" windowWidth="16650" windowHeight="15870" xr2:uid="{46FCF62E-0F38-40EF-B40B-6239A54C7BFA}"/>
+    <workbookView xWindow="3120" yWindow="330" windowWidth="16650" windowHeight="15870" xr2:uid="{46FCF62E-0F38-40EF-B40B-6239A54C7BFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -516,7 +516,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -594,6 +600,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -615,7 +624,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -624,6 +633,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -642,38 +663,17 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1073,13 +1073,13 @@
       <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="56"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="58"/>
       <c r="F2" s="13"/>
       <c r="G2" s="14"/>
       <c r="H2" s="15" t="s">
@@ -1091,19 +1091,19 @@
       <c r="N2" s="2"/>
     </row>
     <row r="3" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="94" t="s">
+      <c r="A3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="95"/>
-      <c r="H3" s="95"/>
-      <c r="I3" s="95"/>
-      <c r="J3" s="95"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="46"/>
       <c r="N3" s="2"/>
     </row>
     <row r="4" spans="1:14" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1124,52 +1124,52 @@
       <c r="A5" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="50" t="s">
+      <c r="B5" s="50"/>
+      <c r="C5" s="50"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="45"/>
-      <c r="I5" s="46"/>
-      <c r="J5" s="46"/>
-      <c r="K5" s="47"/>
+      <c r="G5" s="53"/>
+      <c r="H5" s="47"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="48"/>
+      <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="48"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="50" t="s">
+      <c r="B6" s="50"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="50"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="51"/>
-      <c r="H6" s="45"/>
-      <c r="I6" s="46"/>
-      <c r="J6" s="46"/>
-      <c r="K6" s="47"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="47"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="49"/>
     </row>
     <row r="7" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="50" t="s">
+      <c r="B7" s="51"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="51"/>
+      <c r="E7" s="51"/>
+      <c r="F7" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="51"/>
-      <c r="H7" s="45"/>
-      <c r="I7" s="46"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="47"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
+      <c r="K7" s="49"/>
     </row>
     <row r="8" spans="1:14" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
@@ -1213,103 +1213,103 @@
       <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="44"/>
-      <c r="B11" s="70"/>
-      <c r="C11" s="67" t="s">
+      <c r="A11" s="72"/>
+      <c r="B11" s="73"/>
+      <c r="C11" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="69"/>
+      <c r="D11" s="71"/>
       <c r="E11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="57" t="s">
+      <c r="F11" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="57"/>
-      <c r="H11" s="67" t="s">
+      <c r="G11" s="59"/>
+      <c r="H11" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="I11" s="68"/>
-      <c r="J11" s="68"/>
-      <c r="K11" s="69"/>
+      <c r="I11" s="70"/>
+      <c r="J11" s="70"/>
+      <c r="K11" s="71"/>
     </row>
     <row r="12" spans="1:14" s="4" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="71"/>
-      <c r="B12" s="72"/>
-      <c r="C12" s="86"/>
-      <c r="D12" s="87"/>
-      <c r="E12" s="77"/>
-      <c r="F12" s="58"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="58"/>
-      <c r="I12" s="59"/>
-      <c r="J12" s="59"/>
-      <c r="K12" s="60"/>
+      <c r="A12" s="74"/>
+      <c r="B12" s="75"/>
+      <c r="C12" s="83"/>
+      <c r="D12" s="84"/>
+      <c r="E12" s="80"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="60"/>
+      <c r="I12" s="61"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="62"/>
     </row>
     <row r="13" spans="1:14" s="4" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="73"/>
-      <c r="B13" s="74"/>
-      <c r="C13" s="88"/>
-      <c r="D13" s="89"/>
-      <c r="E13" s="78"/>
-      <c r="F13" s="61"/>
-      <c r="G13" s="63"/>
-      <c r="H13" s="61"/>
-      <c r="I13" s="62"/>
-      <c r="J13" s="62"/>
-      <c r="K13" s="63"/>
+      <c r="A13" s="76"/>
+      <c r="B13" s="77"/>
+      <c r="C13" s="85"/>
+      <c r="D13" s="86"/>
+      <c r="E13" s="81"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="63"/>
+      <c r="I13" s="64"/>
+      <c r="J13" s="64"/>
+      <c r="K13" s="65"/>
     </row>
     <row r="14" spans="1:14" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="73"/>
-      <c r="B14" s="74"/>
-      <c r="C14" s="88"/>
-      <c r="D14" s="89"/>
-      <c r="E14" s="78"/>
-      <c r="F14" s="61"/>
-      <c r="G14" s="63"/>
-      <c r="H14" s="64"/>
-      <c r="I14" s="65"/>
-      <c r="J14" s="65"/>
-      <c r="K14" s="66"/>
+      <c r="A14" s="76"/>
+      <c r="B14" s="77"/>
+      <c r="C14" s="85"/>
+      <c r="D14" s="86"/>
+      <c r="E14" s="81"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="66"/>
+      <c r="I14" s="67"/>
+      <c r="J14" s="67"/>
+      <c r="K14" s="68"/>
     </row>
     <row r="15" spans="1:14" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="73"/>
-      <c r="B15" s="74"/>
-      <c r="C15" s="90"/>
-      <c r="D15" s="91"/>
-      <c r="E15" s="78"/>
-      <c r="F15" s="61"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="58"/>
-      <c r="I15" s="59"/>
-      <c r="J15" s="59"/>
-      <c r="K15" s="60"/>
+      <c r="A15" s="76"/>
+      <c r="B15" s="77"/>
+      <c r="C15" s="93"/>
+      <c r="D15" s="94"/>
+      <c r="E15" s="81"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="60"/>
+      <c r="I15" s="61"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="62"/>
     </row>
     <row r="16" spans="1:14" s="4" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="73"/>
-      <c r="B16" s="74"/>
-      <c r="C16" s="90"/>
-      <c r="D16" s="91"/>
-      <c r="E16" s="78"/>
-      <c r="F16" s="61"/>
-      <c r="G16" s="63"/>
-      <c r="H16" s="61"/>
-      <c r="I16" s="62"/>
-      <c r="J16" s="62"/>
-      <c r="K16" s="63"/>
+      <c r="A16" s="76"/>
+      <c r="B16" s="77"/>
+      <c r="C16" s="93"/>
+      <c r="D16" s="94"/>
+      <c r="E16" s="81"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="63"/>
+      <c r="I16" s="64"/>
+      <c r="J16" s="64"/>
+      <c r="K16" s="65"/>
     </row>
     <row r="17" spans="1:11" s="4" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="75"/>
-      <c r="B17" s="76"/>
-      <c r="C17" s="92"/>
-      <c r="D17" s="93"/>
-      <c r="E17" s="79"/>
-      <c r="F17" s="64"/>
-      <c r="G17" s="66"/>
-      <c r="H17" s="64"/>
-      <c r="I17" s="65"/>
-      <c r="J17" s="65"/>
-      <c r="K17" s="66"/>
+      <c r="A17" s="78"/>
+      <c r="B17" s="79"/>
+      <c r="C17" s="95"/>
+      <c r="D17" s="96"/>
+      <c r="E17" s="82"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="66"/>
+      <c r="I17" s="67"/>
+      <c r="J17" s="67"/>
+      <c r="K17" s="68"/>
     </row>
     <row r="18" spans="1:11" customFormat="1" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1354,10 +1354,10 @@
         <v>22</v>
       </c>
       <c r="G21" s="22"/>
-      <c r="H21" s="85" t="s">
+      <c r="H21" s="92" t="s">
         <v>25</v>
       </c>
-      <c r="I21" s="85"/>
+      <c r="I21" s="92"/>
       <c r="J21" s="22" t="s">
         <v>23</v>
       </c>
@@ -1371,12 +1371,12 @@
       </c>
       <c r="D22" s="40"/>
       <c r="E22" s="11"/>
-      <c r="F22" s="83"/>
-      <c r="G22" s="84"/>
-      <c r="H22" s="83"/>
-      <c r="I22" s="84"/>
-      <c r="J22" s="83"/>
-      <c r="K22" s="80"/>
+      <c r="F22" s="90"/>
+      <c r="G22" s="91"/>
+      <c r="H22" s="90"/>
+      <c r="I22" s="91"/>
+      <c r="J22" s="90"/>
+      <c r="K22" s="87"/>
     </row>
     <row r="23" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="37"/>
@@ -1386,12 +1386,12 @@
       </c>
       <c r="D23" s="40"/>
       <c r="E23" s="11"/>
-      <c r="F23" s="83"/>
-      <c r="G23" s="84"/>
-      <c r="H23" s="83"/>
-      <c r="I23" s="84"/>
-      <c r="J23" s="83"/>
-      <c r="K23" s="80"/>
+      <c r="F23" s="90"/>
+      <c r="G23" s="91"/>
+      <c r="H23" s="90"/>
+      <c r="I23" s="91"/>
+      <c r="J23" s="90"/>
+      <c r="K23" s="87"/>
     </row>
     <row r="24" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="22" t="s">
@@ -1402,10 +1402,10 @@
         <v>4</v>
       </c>
       <c r="D24" s="22"/>
-      <c r="E24" s="82" t="s">
+      <c r="E24" s="89" t="s">
         <v>24</v>
       </c>
-      <c r="F24" s="82"/>
+      <c r="F24" s="89"/>
       <c r="G24" s="22" t="s">
         <v>17</v>
       </c>
@@ -1417,28 +1417,28 @@
     <row r="25" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="25"/>
       <c r="B25" s="25"/>
-      <c r="C25" s="80"/>
-      <c r="D25" s="80"/>
-      <c r="E25" s="81"/>
-      <c r="F25" s="81"/>
-      <c r="G25" s="80"/>
-      <c r="H25" s="80"/>
-      <c r="I25" s="80"/>
-      <c r="J25" s="80"/>
-      <c r="K25" s="80"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="87"/>
+      <c r="E25" s="88"/>
+      <c r="F25" s="88"/>
+      <c r="G25" s="87"/>
+      <c r="H25" s="87"/>
+      <c r="I25" s="87"/>
+      <c r="J25" s="87"/>
+      <c r="K25" s="87"/>
     </row>
     <row r="26" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="25"/>
       <c r="B26" s="25"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="81"/>
-      <c r="F26" s="81"/>
-      <c r="G26" s="80"/>
-      <c r="H26" s="80"/>
-      <c r="I26" s="80"/>
-      <c r="J26" s="80"/>
-      <c r="K26" s="80"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="87"/>
+      <c r="E26" s="88"/>
+      <c r="F26" s="88"/>
+      <c r="G26" s="87"/>
+      <c r="H26" s="87"/>
+      <c r="I26" s="87"/>
+      <c r="J26" s="87"/>
+      <c r="K26" s="87"/>
     </row>
     <row r="27" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="22" t="s">

</xml_diff>